<commit_message>
Bulk product upload: live test run on test.gokesari.com (23/23 pass)
- scripts/test-site/product-import-check.mjs: the live functional run
  (owner, staff and a guarded production smoke mode). Accepts the
  "Import it again?" confirmation and waits for result rows.
- Test report: Test column filled in, new section 2.7 with the 23 live
  cases, regression and APK run numbers; PDF rebuilt.
- Screenshots and raw JSON results from the run.
- Feature README and tracker: Done on Test; production waits for the
  staging -> main release.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tEZLkKWS5b5jdHMF2AcrN
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
@@ -896,7 +896,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="24">
       <c r="A7" s="27" t="inlineStr">
         <is>
@@ -1063,7 +1062,6 @@
       <c r="F13" s="29" t="n"/>
       <c r="G13" s="30" t="n"/>
     </row>
-    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="24">
       <c r="A15" s="27" t="inlineStr">
         <is>
@@ -2295,7 +2293,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -2341,7 +2338,7 @@
       </c>
       <c r="C5" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D5" s="49" t="inlineStr">
@@ -2351,12 +2348,12 @@
       </c>
       <c r="E5" s="49" t="inlineStr">
         <is>
-          <t>Built and unit-tested locally: Template sheet chosen, headings found by content (labels, attribute keys, section headers), ABC123 example + notice rows skipped, key-first mapping with qualifiers stripped (audience kept), repeated #1-#5 columns to arrays, lossless raw cells. 309-column PUZZLES fixture parses in ~0.2 s. Generic: no product-type logic. Not yet on Test.</t>
+          <t>Built and unit-tested locally: Template sheet chosen, headings found by content (labels, attribute keys, section headers), ABC123 example + notice rows skipped, key-first mapping with qualifiers stripped (audience kept), repeated #1-#5 columns to arrays, lossless raw cells. 309-column PUZZLES fixture parses in ~0.2 s. Generic: no product-type logic. Not yet on Test. Live on test.gokesari.com 15 Oct: PI-03 pass (PUZZLES.xlsm: 309 columns, rows 6-7 left out, macros not run).</t>
         </is>
       </c>
       <c r="F5" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2373,7 +2370,7 @@
       </c>
       <c r="C6" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D6" s="49" t="inlineStr">
@@ -2383,12 +2380,12 @@
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>Simple template (Products + Instructions sheets, Barcode Type/Unit/Action dropdowns, EXAMPLE row never imported) and CSV (comma/semicolon/tab, BOM). Header aliases case-insensitive. Tested locally.</t>
+          <t>Simple template (Products + Instructions sheets, Barcode Type/Unit/Action dropdowns, EXAMPLE row never imported) and CSV (comma/semicolon/tab, BOM). Header aliases case-insensitive. Tested locally. Live on test.gokesari.com 15 Oct: PI-02 template download, PI-09 template import pass.</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2405,7 +2402,7 @@
       </c>
       <c r="C7" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
@@ -2415,12 +2412,12 @@
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>All §2 fields mapped; Indian numbers, dd/mm/yyyy and Excel-serial dates, Y/N, units to cm/g. Unreadable values = warnings, raw kept. Decision: file MRP = listing MRP (shop_listing_details), never master.</t>
+          <t>All §2 fields mapped; Indian numbers, dd/mm/yyyy and Excel-serial dates, Y/N, units to cm/g. Unreadable values = warnings, raw kept. Decision: file MRP = listing MRP (shop_listing_details), never master. Live on test.gokesari.com 15 Oct: PI-03/PI-04/PI-09 pass.</t>
         </is>
       </c>
       <c r="F7" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2434,7 @@
       </c>
       <c r="C8" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D8" s="49" t="inlineStr">
@@ -2447,12 +2444,12 @@
       </c>
       <c r="E8" s="49" t="inlineStr">
         <is>
-          <t>SKU (or P-code) → barcode → name+brand(+size/color) → new Pending product. Pending products visible to the existing duplicate check. Decision: fallback category = General (system 'uncategorised').</t>
+          <t>SKU (or P-code) → barcode → name+brand(+size/color) → new Pending product. Pending products visible to the existing duplicate check. Decision: fallback category = General (system 'uncategorised'). Live on test.gokesari.com 15 Oct: PI-05 re-import matched all 5 by SKU (5 updated); PI-11 Edit with no match skipped.</t>
         </is>
       </c>
       <c r="F8" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2469,7 +2466,7 @@
       </c>
       <c r="C9" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D9" s="49" t="inlineStr">
@@ -2479,12 +2476,12 @@
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t>Set / Add modes, blank / negative / non-numeric quantity rules, duplicate-SKU merge, inventory_movements with source=bulk_upload + import_job_id + user, row lock + atomic add (tested with concurrent orders). Online stock.</t>
+          <t>Set / Add modes, blank / negative / non-numeric quantity rules, duplicate-SKU merge, inventory_movements with source=bulk_upload + import_job_id + user, row lock + atomic add (tested with concurrent orders). Online stock. Live on test.gokesari.com 15 Oct: PI-10 Set 11 then Add 4 = 15; PI-11 blank/negative unchanged; PI-13 Delete = stock 0.</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2501,7 +2498,7 @@
       </c>
       <c r="C10" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D10" s="49" t="inlineStr">
@@ -2511,12 +2508,12 @@
       </c>
       <c r="E10" s="49" t="inlineStr">
         <is>
-          <t>Async after commit; http/https only, SSRF guard at connect time, JPEG/PNG/WebP, 5 MB, 15 s, each URL once; existing photo pipeline + moderation; failures are row warnings.</t>
+          <t>Async after commit; http/https only, SSRF guard at connect time, JPEG/PNG/WebP, 5 MB, 15 s, each URL once; existing photo pipeline + moderation; failures are row warnings. Live on test.gokesari.com 15 Oct: Fixture image URLs (example CDN) refused with row warnings, products still created. Real image URLs not tried on the site.</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2533,7 +2530,7 @@
       </c>
       <c r="C11" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D11" s="49" t="inlineStr">
@@ -2543,12 +2540,12 @@
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t>Inventory → Bulk upload (Excel/CSV) tile; /shop/product-import: drag-and-drop, template, help, background check with progress, preview (summary, paginated table, warnings filter, stock mode), import progress, result + report, history, duplicate-file prompt. Checked in a browser locally (screenshots in docs/product-import-2026-10/screenshots).</t>
+          <t>Inventory → Bulk upload (Excel/CSV) tile; /shop/product-import: drag-and-drop, template, help, background check with progress, preview (summary, paginated table, warnings filter, stock mode), import progress, result + report, history, duplicate-file prompt. Checked in a browser locally (screenshots in docs/product-import-2026-10/screenshots). Live on test.gokesari.com 15 Oct: PI-01..PI-15 pass (desktop + phone cards with the Android app agent).</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2565,7 +2562,7 @@
       </c>
       <c r="C12" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D12" s="49" t="inlineStr">
@@ -2575,12 +2572,12 @@
       </c>
       <c r="E12" s="49" t="inlineStr">
         <is>
-          <t>/admin/product-import with shop picker; tiles under admin Product master and operator Catalogue. Checked locally as admin and operator. Operators' prices go to the owner for approval (existing rule).</t>
+          <t>/admin/product-import with shop picker; tiles under admin Product master and operator Catalogue. Checked locally as admin and operator. Operators' prices go to the owner for approval (existing rule). Live on test.gokesari.com 15 Oct: Admin and operator PS-01..04 pass; operator prices go to the owner, admin prices apply.</t>
         </is>
       </c>
       <c r="F12" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2594,7 @@
       </c>
       <c r="C13" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D13" s="49" t="inlineStr">
@@ -2607,12 +2604,12 @@
       </c>
       <c r="E13" s="49" t="inlineStr">
         <is>
-          <t>8 endpoints under /api/v1 (+ shop picker). Owner = own shops only; operator/admin any shop; audit-logged. Route tests pass.</t>
+          <t>8 endpoints under /api/v1 (+ shop picker). Owner = own shops only; operator/admin any shop; audit-logged. Route tests pass. Live on test.gokesari.com 15 Oct: PI-08/PI-09/PI-15 and the staff runs use /api/v1.</t>
         </is>
       </c>
       <c r="F13" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2639,12 +2636,12 @@
       </c>
       <c r="E14" s="49" t="inlineStr">
         <is>
-          <t>Version 1.1.0 / versionCode 2. The app shows the website: the upload uses Android's system document picker (Files, Drive, WhatsApp, e-mail attachments). APKs built by the PR's 'Android APK' workflow; Play Store AAB needs EAS (Expo account) - not run.</t>
+          <t>Version 1.1.0 / versionCode 2. The app shows the website: the upload uses Android's system document picker (Files, Drive, WhatsApp, e-mail attachments). APKs built by the PR's 'Android APK' workflow; Play Store AAB needs EAS (Expo account) - not run. Live on test.gokesari.com 15 Oct: APK run 19 (Android APK workflow) built 1.1.0/versionCode 2; phone-width app agent preview pass (PI-12). System file picker on a real phone not tried; AAB needs EAS.</t>
         </is>
       </c>
       <c r="F14" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2690,7 @@
       </c>
       <c r="C16" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D16" s="49" t="inlineStr">
@@ -2703,12 +2700,12 @@
       </c>
       <c r="E16" s="49" t="inlineStr">
         <is>
-          <t>Event shop.product_import_finished (event layer, no cron) to owner and the operator/admin who ran it; in-app + PUSH queued. Push provider not chosen yet (existing gap).</t>
+          <t>Event shop.product_import_finished (event layer, no cron) to owner and the operator/admin who ran it; in-app + PUSH queued. Push provider not chosen yet (existing gap). Live on test.gokesari.com 15 Oct: PI-14: owner gets 'Bulk product upload finished' in app, also for admin/operator imports. Push: no provider configured.</t>
         </is>
       </c>
       <c r="F16" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2725,7 +2722,7 @@
       </c>
       <c r="C17" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D17" s="49" t="inlineStr">
@@ -2735,12 +2732,12 @@
       </c>
       <c r="E17" s="49" t="inlineStr">
         <is>
-          <t>History list; result report XLSX/CSV (original rows + status + messages); file hash duplicate prompt; 90-day retention purge in the daily seller sweep.</t>
+          <t>History list; result report XLSX/CSV (original rows + status + messages); file hash duplicate prompt; 90-day retention purge in the daily seller sweep. Live on test.gokesari.com 15 Oct: PI-06 report, PI-07 duplicate prompt, PI-08 history pass.</t>
         </is>
       </c>
       <c r="F17" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2754,7 @@
       </c>
       <c r="C18" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D18" s="49" t="inlineStr">
@@ -2767,12 +2764,12 @@
       </c>
       <c r="E18" s="49" t="inlineStr">
         <is>
-          <t>Unit 18 + integration 23 + load 1 (5,000 rows: parse ~2 s, import ~95 s locally) pass; full suite run for regressions (see test report).</t>
+          <t>Unit 18 + integration 23 + load 1 (5,000 rows: parse ~2 s, import ~95 s locally) pass; full suite run for regressions (see test report). Live on test.gokesari.com 15 Oct: 1,811 tests pass locally; CI green on PR #173; live run 23/23 pass.</t>
         </is>
       </c>
       <c r="F18" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2789,7 +2786,7 @@
       </c>
       <c r="C19" s="51" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Done on Test</t>
         </is>
       </c>
       <c r="D19" s="49" t="inlineStr">
@@ -2799,12 +2796,12 @@
       </c>
       <c r="E19" s="49" t="inlineStr">
         <is>
-          <t>Needs the PR merged into staging (owner approval); this session cannot deploy or reach test.gokesari.com. Migration 0077 (after Inventory &amp; Accounting's 0076) is additive.</t>
+          <t>PR #173 merged into staging (2886cf3); test.gokesari.com deployed; Test database run 31 confirms 0077 (80 migrations). Live run 23/23 pass.</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2831,12 +2828,12 @@
       </c>
       <c r="E20" s="49" t="inlineStr">
         <is>
-          <t>After Test sign-off: staging → main (human approval gate). Smoke test plan in the test report.</t>
+          <t>Waiting for the owner's go-ahead: staging -&gt; main also releases #168, #169 and #171 (Inventory &amp; Accounting; its fix PR #172 is still open). Then Production database workflow (migrate) and prod smoke test.</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -2863,12 +2860,12 @@
       </c>
       <c r="E21" s="49" t="inlineStr">
         <is>
-          <t>docs/testing/bulk-product-upload-test-report.md (+ PDF): local results filled in; Test and Prod columns 'Not run' until deployed.</t>
+          <t>Test column filled in (23/23 live pass, section 2.7); Prod column after the production release.</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173 (merged to staging)</t>
         </is>
       </c>
     </row>
@@ -26654,7 +26651,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="30" customHeight="1" s="24">
       <c r="A4" s="28" t="inlineStr">
         <is>
@@ -46124,17 +46120,17 @@
       </c>
       <c r="C45" s="23" t="inlineStr">
         <is>
-          <t>Bulk product upload not deployed</t>
+          <t>Bulk product upload not on production</t>
         </is>
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>Merge the bulk-upload PR into staging (test.gokesari.com), run the environment tests, then staging → main</t>
+          <t>On test.gokesari.com and passing (23/23). Production needs the owner to approve the staging -&gt; main release, which also ships #168, #169, #171; run the Production database workflow first.</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
         <is>
-          <t>BPU-15, BPU-16</t>
+          <t>BPU-16</t>
         </is>
       </c>
       <c r="F45" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Browser document reading (#169): test results on test and production; trackers
- docs/document-upload-2026-10/TEST_RESULTS.md: 14-15 Oct section -
  automated suites, staging before/after (D-18 reproduced, then fields
  pre-filled, engine browser-tesseract), production read-only checks
  (reader files, CSP, the reader run in the browser from gokesari.com's own
  files, branding E2E 18/18). D-18 closed.
- Test results tracker: runs TR-25 (automated), TR-26 (staging), TR-27
  (production) with 22 checks; D-18 fixed; count formulas widened so the
  new rows are counted (27 runs, 362 checks).
- 15 Oct feature status report: NEW-062 and F8.2.6 COMPLETED on
  production; PR register #169 released via #175 / #177, #176 closed;
  decision #41 resolved.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UQBjybK9TNUiDeHR27XPHU
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
@@ -836,7 +836,7 @@
     <row r="2" ht="24" customHeight="1" s="24">
       <c r="A2" s="26" t="inlineStr">
         <is>
-          <t>As of 15 Oct 2026, 06:45 UTC. Production = main @78e7e06 (gokesari.com, migrations to 0075; no code change since 14 Oct). Test site = staging @a3ae8dd (migrations to 0076) - ahead of production by #168, #169 and #171. Open PR: #170 (docs).</t>
+          <t>As of 15 Oct 2026, 06:45 UTC. Production = main @78e7e06 (gokesari.com, migrations to 0075; no code change since 14 Oct). Test site = staging @a3ae8dd (migrations to 0076) - ahead of production by #168, #169 and #171. Open PR: #170 (docs). Updated 15 Oct, 15:00 UTC: #168 and #169 released to gokesari.com (#175, #177).</t>
         </is>
       </c>
     </row>
@@ -861,6 +861,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7" ht="15" customHeight="1" s="24">
       <c r="A7" s="27" t="inlineStr">
         <is>
@@ -1027,6 +1028,7 @@
       <c r="F13" s="29" t="n"/>
       <c r="G13" s="30" t="n"/>
     </row>
+    <row r="14"/>
     <row r="15" ht="15" customHeight="1" s="24">
       <c r="A15" s="27" t="inlineStr">
         <is>
@@ -2172,7 +2174,7 @@
     <row r="85" ht="36" customHeight="1" s="24">
       <c r="A85" s="39" t="inlineStr">
         <is>
-          <t>3. Document auto-read (NEW-062) now works on test by reading the photo in the owner's browser (#169) - this removes the need to send KYC documents to Claude. Release it to fix production.</t>
+          <t>3. Document auto-read (NEW-062) works on gokesari.com since 15 Oct: the owner's browser reads the photo (#169, released via #175 / #177), so no KYC document needs to go to Claude. Verified on test (fields pre-filled) and production (read-only checks).</t>
         </is>
       </c>
     </row>
@@ -2206,19 +2208,19 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A84:G84"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="A89:G89"/>
+    <mergeCell ref="A88:G88"/>
     <mergeCell ref="E13:G13"/>
+    <mergeCell ref="E11:G11"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A83:G83"/>
+    <mergeCell ref="A87:G87"/>
     <mergeCell ref="A4:G4"/>
+    <mergeCell ref="E8:G8"/>
     <mergeCell ref="E9:G9"/>
-    <mergeCell ref="E11:G11"/>
-    <mergeCell ref="A83:G83"/>
-    <mergeCell ref="A88:G88"/>
-    <mergeCell ref="A87:G87"/>
     <mergeCell ref="E12:G12"/>
-    <mergeCell ref="A84:G84"/>
-    <mergeCell ref="A89:G89"/>
-    <mergeCell ref="A3:G3"/>
-    <mergeCell ref="E8:G8"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A86:G86"/>
     <mergeCell ref="A85:G85"/>
@@ -21140,47 +21142,47 @@
       </c>
       <c r="I210" s="32" t="inlineStr">
         <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="J210" s="34" t="inlineStr">
+        <is>
+          <t>Production (gokesari.com)</t>
+        </is>
+      </c>
+      <c r="K210" s="34" t="inlineStr">
+        <is>
+          <t>Live - rule documentUpload.enabled = on; photos read in the owner's browser (DOCUMENT_OCR_BROWSER on by default; 'off' = server only)</t>
+        </is>
+      </c>
+      <c r="L210" s="34" t="inlineStr">
+        <is>
+          <t>#146; #147 (25 s limit, 'type the details', health check); #148 (OCR engine shipped); #169 (photos read in the owner's browser)</t>
+        </is>
+      </c>
+      <c r="M210" s="34" t="inlineStr">
+        <is>
+          <t>#149; #175 (#169 cherry-picked); #177 (same commit, no change)</t>
+        </is>
+      </c>
+      <c r="N210" s="34" t="inlineStr">
+        <is>
+          <t>Scanned PDFs without a text layer still ask for a photo. iOS before 16 falls back to the server reader (owner types the details). No real owner upload on production recorded yet</t>
+        </is>
+      </c>
+      <c r="O210" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P210" s="34" t="inlineStr">
+        <is>
           <t>IN PROGRESS</t>
         </is>
       </c>
-      <c r="J210" s="34" t="inlineStr">
-        <is>
-          <t>Production - partly live</t>
-        </is>
-      </c>
-      <c r="K210" s="34" t="inlineStr">
-        <is>
-          <t>Rule documentUpload.enabled = on; DOCUMENT_OCR_PROVIDER = tesseract; reading times out after 25 s and the owner types the details</t>
-        </is>
-      </c>
-      <c r="L210" s="34" t="inlineStr">
-        <is>
-          <t>#146; #147 (25 s limit, 'type the details', health check); #148 (OCR engine shipped)</t>
-        </is>
-      </c>
-      <c r="M210" s="34" t="inlineStr">
-        <is>
-          <t>#149</t>
-        </is>
-      </c>
-      <c r="N210" s="34" t="inlineStr">
-        <is>
-          <t>On test, the owner's browser now reads the photo (#169), so auto-read works there; production still has owners type the details until #169 is released. iPhones older than iOS 16 fall back to the server reader</t>
-        </is>
-      </c>
-      <c r="O210" s="34" t="inlineStr">
-        <is>
-          <t>Release #169 to gokesari.com and record a real photo read on production (Blockers #41)</t>
-        </is>
-      </c>
-      <c r="P210" s="34" t="inlineStr">
-        <is>
-          <t>IN PROGRESS</t>
-        </is>
-      </c>
       <c r="Q210" s="34" t="inlineStr">
         <is>
-          <t>#169 (test site, 14 Oct): the photo is read in the owner's browser (tesseract.js, files served from our own site, nothing sent elsewhere); the server re-checks the text. Fixes D-18 on test without sending KYC documents to Claude. Checked 15 Oct: test.gokesari.com/api/ocr-assets/7.0.0/worker.min.js 200, gokesari.com 404 (not released).</t>
+          <t>#169: photos read in the owner's browser (fixes D-18). Verified on test (15 Oct: fields pre-filled, engine browser-tesseract 92 %) and released 15 Oct (#175 / #177; production read-only checks PASS)</t>
         </is>
       </c>
       <c r="R210" s="34" t="inlineStr">
@@ -31294,17 +31296,17 @@
       <c r="F132" s="32" t="n"/>
       <c r="G132" s="32" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="H132" s="34" t="inlineStr">
         <is>
-          <t>#146-#149; #169</t>
+          <t>#146-#149; #169; #175</t>
         </is>
       </c>
       <c r="I132" s="34" t="inlineStr">
         <is>
-          <t>On test the owner's browser reads the photo (#169); production still has owners type the details until #169 is released</t>
+          <t>Live on gokesari.com since 15 Oct: the owner's browser reads the photo and pre-fills the details</t>
         </is>
       </c>
     </row>
@@ -34536,7 +34538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L172"/>
+  <dimension ref="A1:L174"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="23" min="1" max="1"/>
@@ -44390,17 +44392,17 @@
       </c>
       <c r="J170" s="34" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NEW-062</t>
         </is>
       </c>
       <c r="K170" s="34" t="inlineStr">
         <is>
-          <t>Not yet (test site only)</t>
+          <t>#175 (cherry-pick); #177</t>
         </is>
       </c>
       <c r="L170" s="34" t="inlineStr">
         <is>
-          <t>CSP adds 'wasm-unsafe-eval'; switch DOCUMENT_OCR_BROWSER=off goes back to server-only.</t>
+          <t>CSP adds 'wasm-unsafe-eval'; switch DOCUMENT_OCR_BROWSER=off goes back to server-only. Verified on test 15 Oct (TR-26).</t>
         </is>
       </c>
     </row>
@@ -44521,6 +44523,126 @@
       <c r="L172" s="34" t="inlineStr">
         <is>
           <t>Migration 0076 (24 tables, additive; rollback-0076.sql).</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="46" t="n">
+        <v>176</v>
+      </c>
+      <c r="B173" s="34" t="inlineStr">
+        <is>
+          <t>Release: document photos read in the owner's browser (#169)</t>
+        </is>
+      </c>
+      <c r="C173" s="34" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D173" s="34" t="inlineStr">
+        <is>
+          <t>staging -&gt; main</t>
+        </is>
+      </c>
+      <c r="E173" s="34" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F173" s="34" t="inlineStr">
+        <is>
+          <t>Closed - not merged</t>
+        </is>
+      </c>
+      <c r="G173" s="34" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H173" s="34" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I173" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J173" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K173" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L173" s="34" t="inlineStr">
+        <is>
+          <t>Closed: staging also carried #168, #171 (migration 0076) and #173 (migration 0077), not approved for release here. Replaced by #177.</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="46" t="n">
+        <v>177</v>
+      </c>
+      <c r="B174" s="34" t="inlineStr">
+        <is>
+          <t>Release: document photos read in the owner's browser (#169, fixes D-18)</t>
+        </is>
+      </c>
+      <c r="C174" s="34" t="inlineStr">
+        <is>
+          <t>Release (branch -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D174" s="34" t="inlineStr">
+        <is>
+          <t>claude/gracious-einstein-24qjjh -&gt; main</t>
+        </is>
+      </c>
+      <c r="E174" s="34" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F174" s="34" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G174" s="34" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H174" s="34" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I174" s="34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J174" s="34" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="K174" s="34" t="inlineStr">
+        <is>
+          <t>Itself (merged to main)</t>
+        </is>
+      </c>
+      <c r="L174" s="34" t="inlineStr">
+        <is>
+          <t>Same commit as #175's cherry-pick of #169, merged after it: no code change. Production checks 15 Oct (TR-27) PASS.</t>
         </is>
       </c>
     </row>
@@ -46397,7 +46519,7 @@
       </c>
       <c r="D42" s="34" t="inlineStr">
         <is>
-          <t>Update 15 Oct: #169 reads the photo in the owner's browser (no document leaves the device to be read), working on test. Releasing #169 removes the need to decide on Claude for KYC documents. Before: The local OCR worker does not start on Hostinger (owners type the details). Either fix tesseract's start, or allow DOCUMENT_OCR_PROVIDER=claude - KYC documents would go to Anthropic (DPA / privacy decision).</t>
+          <t>Resolved 15 Oct: #169 reads the photo in the owner's browser (no document leaves the device to be read); released to gokesari.com (#175 / #177) and verified on test and production. No decision on Claude for KYC documents is needed. Before: the local OCR worker did not start on Hostinger.</t>
         </is>
       </c>
       <c r="E42" s="34" t="inlineStr">
@@ -46412,7 +46534,7 @@
       </c>
       <c r="G42" s="34" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="H42" s="34" t="inlineStr">
@@ -46597,7 +46719,7 @@
       </c>
       <c r="D47" s="34" t="inlineStr">
         <is>
-          <t>Staging is ahead of main by the shop switcher (#168), browser document reading (#169) and Inventory &amp; Accounting (#171, migration 0076). #168 and #169 are ready; #171 waits on #45.</t>
+          <t>Staging is ahead of main by the shop switcher (#168), browser document reading (#169) and Inventory &amp; Accounting (#171, migration 0076). #168 and #169 are ready; #171 waits on #45. Update 15 Oct: #168 and #169 released to gokesari.com (#175; #177 for #169). #171 and #173 remain on staging.</t>
         </is>
       </c>
       <c r="E47" s="34" t="inlineStr">

</xml_diff>

<commit_message>
Bulk product upload: production results (gokesari.com, release #179)
- Test report: Production deployed 15 Oct 15:58 UTC; new section 2.8,
  signed-out production smoke 13/13 pass (bulk upload pages and API,
  Inventory & Accounting smoke 11/11); PDF rebuilt.
- README and the 15 Oct tracker: Done on Prod; open items are a
  signed-in import on a named production test shop and the Production
  database workflow's repository variables.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016tEZLkKWS5b5jdHMF2AcrN
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
@@ -2324,7 +2324,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="48" t="inlineStr">
         <is>
@@ -2370,7 +2369,7 @@
       </c>
       <c r="C5" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D5" s="49" t="inlineStr">
@@ -2380,12 +2379,12 @@
       </c>
       <c r="E5" s="49" t="inlineStr">
         <is>
-          <t>Built and unit-tested locally: Template sheet chosen, headings found by content (labels, attribute keys, section headers), ABC123 example + notice rows skipped, key-first mapping with qualifiers stripped (audience kept), repeated #1-#5 columns to arrays, lossless raw cells. 309-column PUZZLES fixture parses in ~0.2 s. Generic: no product-type logic. Not yet on Test. Live on test.gokesari.com 15 Oct: PI-03 pass (PUZZLES.xlsm: 309 columns, rows 6-7 left out, macros not run).</t>
+          <t>Built and unit-tested locally: Template sheet chosen, headings found by content (labels, attribute keys, section headers), ABC123 example + notice rows skipped, key-first mapping with qualifiers stripped (audience kept), repeated #1-#5 columns to arrays, lossless raw cells. 309-column PUZZLES fixture parses in ~0.2 s. Generic: no product-type logic. Not yet on Test. Live on test.gokesari.com 15 Oct: PI-03 pass (PUZZLES.xlsm: 309 columns, rows 6-7 left out, macros not run). Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F5" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2402,7 +2401,7 @@
       </c>
       <c r="C6" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D6" s="49" t="inlineStr">
@@ -2412,12 +2411,12 @@
       </c>
       <c r="E6" s="49" t="inlineStr">
         <is>
-          <t>Simple template (Products + Instructions sheets, Barcode Type/Unit/Action dropdowns, EXAMPLE row never imported) and CSV (comma/semicolon/tab, BOM). Header aliases case-insensitive. Tested locally. Live on test.gokesari.com 15 Oct: PI-02 template download, PI-09 template import pass.</t>
+          <t>Simple template (Products + Instructions sheets, Barcode Type/Unit/Action dropdowns, EXAMPLE row never imported) and CSV (comma/semicolon/tab, BOM). Header aliases case-insensitive. Tested locally. Live on test.gokesari.com 15 Oct: PI-02 template download, PI-09 template import pass. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F6" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2433,7 @@
       </c>
       <c r="C7" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D7" s="49" t="inlineStr">
@@ -2444,12 +2443,12 @@
       </c>
       <c r="E7" s="49" t="inlineStr">
         <is>
-          <t>All §2 fields mapped; Indian numbers, dd/mm/yyyy and Excel-serial dates, Y/N, units to cm/g. Unreadable values = warnings, raw kept. Decision: file MRP = listing MRP (shop_listing_details), never master. Live on test.gokesari.com 15 Oct: PI-03/PI-04/PI-09 pass.</t>
+          <t>All §2 fields mapped; Indian numbers, dd/mm/yyyy and Excel-serial dates, Y/N, units to cm/g. Unreadable values = warnings, raw kept. Decision: file MRP = listing MRP (shop_listing_details), never master. Live on test.gokesari.com 15 Oct: PI-03/PI-04/PI-09 pass. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F7" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2466,7 +2465,7 @@
       </c>
       <c r="C8" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D8" s="49" t="inlineStr">
@@ -2476,12 +2475,12 @@
       </c>
       <c r="E8" s="49" t="inlineStr">
         <is>
-          <t>SKU (or P-code) → barcode → name+brand(+size/color) → new Pending product. Pending products visible to the existing duplicate check. Decision: fallback category = General (system 'uncategorised'). Live on test.gokesari.com 15 Oct: PI-05 re-import matched all 5 by SKU (5 updated); PI-11 Edit with no match skipped.</t>
+          <t>SKU (or P-code) → barcode → name+brand(+size/color) → new Pending product. Pending products visible to the existing duplicate check. Decision: fallback category = General (system 'uncategorised'). Live on test.gokesari.com 15 Oct: PI-05 re-import matched all 5 by SKU (5 updated); PI-11 Edit with no match skipped. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F8" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2498,7 +2497,7 @@
       </c>
       <c r="C9" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D9" s="49" t="inlineStr">
@@ -2508,12 +2507,12 @@
       </c>
       <c r="E9" s="49" t="inlineStr">
         <is>
-          <t>Set / Add modes, blank / negative / non-numeric quantity rules, duplicate-SKU merge, inventory_movements with source=bulk_upload + import_job_id + user, row lock + atomic add (tested with concurrent orders). Online stock. Live on test.gokesari.com 15 Oct: PI-10 Set 11 then Add 4 = 15; PI-11 blank/negative unchanged; PI-13 Delete = stock 0.</t>
+          <t>Set / Add modes, blank / negative / non-numeric quantity rules, duplicate-SKU merge, inventory_movements with source=bulk_upload + import_job_id + user, row lock + atomic add (tested with concurrent orders). Online stock. Live on test.gokesari.com 15 Oct: PI-10 Set 11 then Add 4 = 15; PI-11 blank/negative unchanged; PI-13 Delete = stock 0. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F9" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2529,7 @@
       </c>
       <c r="C10" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D10" s="49" t="inlineStr">
@@ -2540,12 +2539,12 @@
       </c>
       <c r="E10" s="49" t="inlineStr">
         <is>
-          <t>Async after commit; http/https only, SSRF guard at connect time, JPEG/PNG/WebP, 5 MB, 15 s, each URL once; existing photo pipeline + moderation; failures are row warnings. Live on test.gokesari.com 15 Oct: Fixture image URLs (example CDN) refused with row warnings, products still created. Real image URLs not tried on the site.</t>
+          <t>Async after commit; http/https only, SSRF guard at connect time, JPEG/PNG/WebP, 5 MB, 15 s, each URL once; existing photo pipeline + moderation; failures are row warnings. Live on test.gokesari.com 15 Oct: Fixture image URLs (example CDN) refused with row warnings, products still created. Real image URLs not tried on the site. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F10" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2562,7 +2561,7 @@
       </c>
       <c r="C11" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D11" s="49" t="inlineStr">
@@ -2572,12 +2571,12 @@
       </c>
       <c r="E11" s="49" t="inlineStr">
         <is>
-          <t>Inventory → Bulk upload (Excel/CSV) tile; /shop/product-import: drag-and-drop, template, help, background check with progress, preview (summary, paginated table, warnings filter, stock mode), import progress, result + report, history, duplicate-file prompt. Checked in a browser locally (screenshots in docs/product-import-2026-10/screenshots). Live on test.gokesari.com 15 Oct: PI-01..PI-15 pass (desktop + phone cards with the Android app agent).</t>
+          <t>Inventory → Bulk upload (Excel/CSV) tile; /shop/product-import: drag-and-drop, template, help, background check with progress, preview (summary, paginated table, warnings filter, stock mode), import progress, result + report, history, duplicate-file prompt. Checked in a browser locally (screenshots in docs/product-import-2026-10/screenshots). Live on test.gokesari.com 15 Oct: PI-01..PI-15 pass (desktop + phone cards with the Android app agent). Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F11" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2594,7 +2593,7 @@
       </c>
       <c r="C12" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D12" s="49" t="inlineStr">
@@ -2604,12 +2603,12 @@
       </c>
       <c r="E12" s="49" t="inlineStr">
         <is>
-          <t>/admin/product-import with shop picker; tiles under admin Product master and operator Catalogue. Checked locally as admin and operator. Operators' prices go to the owner for approval (existing rule). Live on test.gokesari.com 15 Oct: Admin and operator PS-01..04 pass; operator prices go to the owner, admin prices apply.</t>
+          <t>/admin/product-import with shop picker; tiles under admin Product master and operator Catalogue. Checked locally as admin and operator. Operators' prices go to the owner for approval (existing rule). Live on test.gokesari.com 15 Oct: Admin and operator PS-01..04 pass; operator prices go to the owner, admin prices apply. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F12" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2626,7 +2625,7 @@
       </c>
       <c r="C13" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D13" s="49" t="inlineStr">
@@ -2636,12 +2635,12 @@
       </c>
       <c r="E13" s="49" t="inlineStr">
         <is>
-          <t>8 endpoints under /api/v1 (+ shop picker). Owner = own shops only; operator/admin any shop; audit-logged. Route tests pass. Live on test.gokesari.com 15 Oct: PI-08/PI-09/PI-15 and the staff runs use /api/v1.</t>
+          <t>8 endpoints under /api/v1 (+ shop picker). Owner = own shops only; operator/admin any shop; audit-logged. Route tests pass. Live on test.gokesari.com 15 Oct: PI-08/PI-09/PI-15 and the staff runs use /api/v1. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F13" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2673,7 +2672,7 @@
       </c>
       <c r="F14" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2705,7 +2704,7 @@
       </c>
       <c r="F15" s="49" t="inlineStr">
         <is>
-          <t>claude/amazing-ritchie-9vlq9f</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2722,7 +2721,7 @@
       </c>
       <c r="C16" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D16" s="49" t="inlineStr">
@@ -2732,12 +2731,12 @@
       </c>
       <c r="E16" s="49" t="inlineStr">
         <is>
-          <t>Event shop.product_import_finished (event layer, no cron) to owner and the operator/admin who ran it; in-app + PUSH queued. Push provider not chosen yet (existing gap). Live on test.gokesari.com 15 Oct: PI-14: owner gets 'Bulk product upload finished' in app, also for admin/operator imports. Push: no provider configured.</t>
+          <t>Event shop.product_import_finished (event layer, no cron) to owner and the operator/admin who ran it; in-app + PUSH queued. Push provider not chosen yet (existing gap). Live on test.gokesari.com 15 Oct: PI-14: owner gets 'Bulk product upload finished' in app, also for admin/operator imports. Push: no provider configured. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F16" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2753,7 @@
       </c>
       <c r="C17" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D17" s="49" t="inlineStr">
@@ -2764,12 +2763,12 @@
       </c>
       <c r="E17" s="49" t="inlineStr">
         <is>
-          <t>History list; result report XLSX/CSV (original rows + status + messages); file hash duplicate prompt; 90-day retention purge in the daily seller sweep. Live on test.gokesari.com 15 Oct: PI-06 report, PI-07 duplicate prompt, PI-08 history pass.</t>
+          <t>History list; result report XLSX/CSV (original rows + status + messages); file hash duplicate prompt; 90-day retention purge in the daily seller sweep. Live on test.gokesari.com 15 Oct: PI-06 report, PI-07 duplicate prompt, PI-08 history pass. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F17" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2786,7 +2785,7 @@
       </c>
       <c r="C18" s="50" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D18" s="49" t="inlineStr">
@@ -2796,12 +2795,12 @@
       </c>
       <c r="E18" s="49" t="inlineStr">
         <is>
-          <t>Unit 18 + integration 23 + load 1 (5,000 rows: parse ~2 s, import ~95 s locally) pass; full suite run for regressions (see test report). Live on test.gokesari.com 15 Oct: 1,811 tests pass locally; CI green on PR #173; live run 23/23 pass.</t>
+          <t>Unit 18 + integration 23 + load 1 (5,000 rows: parse ~2 s, import ~95 s locally) pass; full suite run for regressions (see test report). Live on test.gokesari.com 15 Oct: 1,811 tests pass locally; CI green on PR #173; live run 23/23 pass. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F18" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2818,7 +2817,7 @@
       </c>
       <c r="C19" s="51" t="inlineStr">
         <is>
-          <t>Done on Test</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D19" s="49" t="inlineStr">
@@ -2828,12 +2827,12 @@
       </c>
       <c r="E19" s="49" t="inlineStr">
         <is>
-          <t>PR #173 merged into staging (2886cf3); test.gokesari.com deployed; Test database run 31 confirms 0077 (80 migrations). Live run 23/23 pass.</t>
+          <t>PR #173 merged into staging (2886cf3); test.gokesari.com deployed; Test database run 31 confirms 0077 (80 migrations). Live run 23/23 pass. Released to gokesari.com 15 Oct 15:58 UTC (PR #179); signed-out prod checks pass.</t>
         </is>
       </c>
       <c r="F19" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2850,7 +2849,7 @@
       </c>
       <c r="C20" s="51" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D20" s="49" t="inlineStr">
@@ -2860,12 +2859,12 @@
       </c>
       <c r="E20" s="49" t="inlineStr">
         <is>
-          <t>Waiting for the owner's go-ahead: staging -&gt; main also releases #168, #169 and #171 (Inventory &amp; Accounting; its fix PR #172 is still open). Then Production database workflow (migrate) and prod smoke test.</t>
+          <t>Release PR #179 merged to main (acfaa6a); Hostinger build applied migrations 0076-0078 (MIGRATE_ON_BUILD) and gokesari.com went live 15:58 UTC. Signed-out smoke 13/13 pass. Signed-in import on prod not run (no designated test shop). The Production database workflow needs PROD_DATABASE_HOST / PROD_DATABASE_NAME / TEST_DATABASE_HOST repository variables (owner).</t>
         </is>
       </c>
       <c r="F20" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -2882,7 +2881,7 @@
       </c>
       <c r="C21" s="50" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done on Prod</t>
         </is>
       </c>
       <c r="D21" s="49" t="inlineStr">
@@ -2892,12 +2891,12 @@
       </c>
       <c r="E21" s="49" t="inlineStr">
         <is>
-          <t>Test column filled in (23/23 live pass, section 2.7); Prod column after the production release.</t>
+          <t>Test report md + PDF: Test 23/23 (section 2.7), Prod signed-out 13/13 (section 2.8).</t>
         </is>
       </c>
       <c r="F21" s="49" t="inlineStr">
         <is>
-          <t>PR #173 (merged to staging)</t>
+          <t>PR #173, #174, release #179</t>
         </is>
       </c>
     </row>
@@ -47280,12 +47279,12 @@
       </c>
       <c r="C48" s="23" t="inlineStr">
         <is>
-          <t>Bulk product upload not on production</t>
+          <t>Bulk product upload: production checks signed in</t>
         </is>
       </c>
       <c r="D48" s="23" t="inlineStr">
         <is>
-          <t>On test.gokesari.com and passing (23/23). Production needs the owner to approve the staging -&gt; main release, which also ships #168, #169, #171; run the Production database workflow first.</t>
+          <t>Live on gokesari.com since 15 Oct 15:58 UTC (#179). A signed-in import on production needs a designated test shop; the Production database workflow needs its repository variables set.</t>
         </is>
       </c>
       <c r="E48" s="23" t="inlineStr">

</xml_diff>

<commit_message>
Feature and product status 18 Oct 2026
- docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-18.xlsx: the
  16 Oct report rolled forward with PRs #185-#188. #184 (PMD loader race
  fix) is now on gokesari.com via #185, Blockers #56 resolved; #178 was
  merged on 15 Oct, not an open draft; #185-#188 added to the PR register.
  No feature changed status: 227 of 267 completed (85 %).
- open-features.xlsx: replaces the 3 Oct snapshot. Summary, a Products
  sheet (14 products / modules with status and open feature IDs), every
  open feature, the full feature list, pending decisions and open go-live
  blockers, all taken from the 18 Oct report.
- Carries the 15 Oct evening and 16 Oct workbooks from the unmerged #183.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HxHwkpvWSuYNUgUzytqbQ6
</commit_message>
<xml_diff>
--- a/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
+++ b/docs/gokesari-audit/GOKESARI_FEATURE_STATUS_REPORT_2026-10-15.xlsx
@@ -19,9 +19,9 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Feature Register'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Process Flow Tree'!$A$4:$I$217</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Process Flow Tree'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PR Register'!$A$1:$L$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'PR Register'!$A$1:$L$183</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="5">'PR Register'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Blockers &amp; Decisions'!$A$1:$H$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Blockers &amp; Decisions'!$A$1:$H$57</definedName>
   </definedNames>
   <calcPr calcId="171027" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -105,21 +105,6 @@
     <font>
       <name val="Arial"/>
       <charset val="1"/>
-      <b val="1"/>
-      <color rgb="FF1D4ED8"/>
-      <sz val="9"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="0"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <charset val="1"/>
-      <family val="0"/>
       <b val="1"/>
       <color rgb="FF1D4ED8"/>
       <sz val="9"/>
@@ -256,7 +241,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
@@ -350,18 +335,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="general" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -987,7 +960,7 @@
     <row r="2" ht="24" customFormat="1" customHeight="1" s="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>As of 15 Oct 2026, 16:10 UTC. Production = main @acfaa6a (gokesari.com, migrations to 0078): release #179 put Inventory &amp; Accounting (#171, #172) and bulk product upload (#173, #174) live; #168 and #169 were released earlier the same day (#175, #177). Test site = staging (same code). Sub-feature sheets: "Bulk Product Upload" and "Inventory &amp; Accounting".</t>
+          <t>As of 15 Oct 2026, 16:45 UTC. Production = main @acfaa6a (gokesari.com, migrations to 0078): release #179 put Inventory &amp; Accounting (#171, #172) and bulk product upload (#173, #174) live; #168 and #169 were released earlier the same day (#175, #177). Test site = staging (same code). Sub-feature sheets: "Bulk Product Upload" and "Inventory &amp; Accounting". Shop switcher (NEW-066) and browser document reading (NEW-062) marked COMPLETED after release #175 (live 14:43 UTC); PR register to #182 (#178 open).</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2057,7 @@
         </is>
       </c>
       <c r="B61" s="10">
-        <f>COUNTIF('PR Register'!$F$2:$F$172,A61)</f>
+        <f>COUNTIF('PR Register'!$F$2:$F$183,A61)</f>
         <v/>
       </c>
     </row>
@@ -2095,7 +2068,7 @@
         </is>
       </c>
       <c r="B62" s="10">
-        <f>COUNTIF('PR Register'!$F$2:$F$172,A62)</f>
+        <f>COUNTIF('PR Register'!$F$2:$F$183,A62)</f>
         <v/>
       </c>
     </row>
@@ -2106,7 +2079,7 @@
         </is>
       </c>
       <c r="B63" s="10">
-        <f>COUNTIF('PR Register'!$F$2:$F$172,A63)</f>
+        <f>COUNTIF('PR Register'!$F$2:$F$183,A63)</f>
         <v/>
       </c>
     </row>
@@ -2117,7 +2090,7 @@
         </is>
       </c>
       <c r="B64" s="10">
-        <f>COUNTIF('PR Register'!$F$2:$F$172,A64)</f>
+        <f>COUNTIF('PR Register'!$F$2:$F$183,A64)</f>
         <v/>
       </c>
     </row>
@@ -2151,7 +2124,7 @@
         </is>
       </c>
       <c r="B67" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A67)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A67)</f>
         <v/>
       </c>
     </row>
@@ -2162,7 +2135,7 @@
         </is>
       </c>
       <c r="B68" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A68)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A68)</f>
         <v/>
       </c>
     </row>
@@ -2173,7 +2146,7 @@
         </is>
       </c>
       <c r="B69" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A69)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A69)</f>
         <v/>
       </c>
     </row>
@@ -2184,7 +2157,7 @@
         </is>
       </c>
       <c r="B70" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A70)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A70)</f>
         <v/>
       </c>
     </row>
@@ -2195,7 +2168,7 @@
         </is>
       </c>
       <c r="B71" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A71)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A71)</f>
         <v/>
       </c>
     </row>
@@ -2206,7 +2179,7 @@
         </is>
       </c>
       <c r="B72" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A72)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A72)</f>
         <v/>
       </c>
     </row>
@@ -2217,7 +2190,7 @@
         </is>
       </c>
       <c r="B73" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A73)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A73)</f>
         <v/>
       </c>
     </row>
@@ -2228,7 +2201,7 @@
         </is>
       </c>
       <c r="B74" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A74)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A74)</f>
         <v/>
       </c>
     </row>
@@ -2239,7 +2212,7 @@
         </is>
       </c>
       <c r="B75" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A75)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A75)</f>
         <v/>
       </c>
     </row>
@@ -2250,7 +2223,7 @@
         </is>
       </c>
       <c r="B76" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A76)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A76)</f>
         <v/>
       </c>
     </row>
@@ -2261,7 +2234,7 @@
         </is>
       </c>
       <c r="B77" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A77)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A77)</f>
         <v/>
       </c>
     </row>
@@ -2272,7 +2245,7 @@
         </is>
       </c>
       <c r="B78" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A78)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A78)</f>
         <v/>
       </c>
     </row>
@@ -2283,7 +2256,7 @@
         </is>
       </c>
       <c r="B79" s="10">
-        <f>COUNTIF('PR Register'!$C$2:$C$172,A79)</f>
+        <f>COUNTIF('PR Register'!$C$2:$C$183,A79)</f>
         <v/>
       </c>
     </row>
@@ -2321,9 +2294,9 @@
       </c>
     </row>
     <row r="85" ht="36" customFormat="1" customHeight="1" s="2">
-      <c r="A85" s="37" t="inlineStr">
-        <is>
-          <t>3. Document auto-read (NEW-062) works on gokesari.com since 15 Oct: the owner's browser reads the photo (#169, released via #175 / #177), so no KYC document needs to go to Claude. Verified on test (fields pre-filled) and production (read-only checks).</t>
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>3. Document auto-read (NEW-062) now works on gokesari.com: the owner's browser reads the photo (#169, released by #175 at 14:43 UTC), so KYC documents are not sent to Claude. Production check PASS (licence number and expiry at 91 %); watch the first real upload. Blockers #41 resolved.</t>
         </is>
       </c>
     </row>
@@ -24687,37 +24660,37 @@
           <t>-</t>
         </is>
       </c>
-      <c r="I210" s="38" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="J210" s="39" t="inlineStr">
+      <c r="I210" s="10" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="J210" s="12" t="inlineStr">
         <is>
           <t>Production (gokesari.com)</t>
         </is>
       </c>
-      <c r="K210" s="39" t="inlineStr">
+      <c r="K210" s="12" t="inlineStr">
         <is>
           <t>Live - rule documentUpload.enabled = on; photos read in the owner's browser (DOCUMENT_OCR_BROWSER on by default; 'off' = server only)</t>
         </is>
       </c>
-      <c r="L210" s="39" t="inlineStr">
+      <c r="L210" s="12" t="inlineStr">
         <is>
           <t>#146; #147 (25 s limit, 'type the details', health check); #148 (OCR engine shipped); #169 (photos read in the owner's browser)</t>
         </is>
       </c>
-      <c r="M210" s="39" t="inlineStr">
+      <c r="M210" s="12" t="inlineStr">
         <is>
           <t>#149; #175 (#169 cherry-picked); #177 (same commit, no change)</t>
         </is>
       </c>
-      <c r="N210" s="39" t="inlineStr">
+      <c r="N210" s="12" t="inlineStr">
         <is>
           <t>Scanned PDFs without a text layer still ask for a photo. iOS before 16 falls back to the server reader (owner types the details). No real owner upload on production recorded yet</t>
         </is>
       </c>
-      <c r="O210" s="39" t="inlineStr">
+      <c r="O210" s="12" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -24727,14 +24700,14 @@
           <t>IN PROGRESS</t>
         </is>
       </c>
-      <c r="Q210" s="39" t="inlineStr">
+      <c r="Q210" s="12" t="inlineStr">
         <is>
           <t>#169: photos read in the owner's browser (fixes D-18). Verified on test (15 Oct: fields pre-filled, engine browser-tesseract 92 %) and released 15 Oct (#175 / #177; production read-only checks PASS)</t>
         </is>
       </c>
       <c r="R210" s="12" t="inlineStr">
         <is>
-          <t>docs/document-upload-2026-10/README.md; TEST_RESULTS.md; drizzle/0075_seller_document_uploads.sql</t>
+          <t>docs/document-upload-2026-10/TEST_RESULTS.md (PR #178)</t>
         </is>
       </c>
     </row>
@@ -25049,17 +25022,17 @@
       </c>
       <c r="I214" s="10" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="J214" s="12" t="inlineStr">
         <is>
-          <t>Test site only (test.gokesari.com)</t>
+          <t>Production (gokesari.com)</t>
         </is>
       </c>
       <c r="K214" s="12" t="inlineStr">
         <is>
-          <t>Live on test (no rule)</t>
+          <t>Live (no rule)</t>
         </is>
       </c>
       <c r="L214" s="12" t="inlineStr">
@@ -25069,17 +25042,17 @@
       </c>
       <c r="M214" s="12" t="inlineStr">
         <is>
-          <t>Not yet (test site only)</t>
+          <t>#175 (15 Oct, live 14:43 UTC)</t>
         </is>
       </c>
       <c r="N214" s="12" t="inlineStr">
         <is>
-          <t>Release to gokesari.com</t>
+          <t>Not yet seen signed in on production (needs an owner with two or more shops)</t>
         </is>
       </c>
       <c r="O214" s="12" t="inlineStr">
         <is>
-          <t>Release staging -&gt; main (Blockers #46)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="P214" s="12" t="inlineStr">
@@ -25089,7 +25062,7 @@
       </c>
       <c r="Q214" s="12" t="inlineStr">
         <is>
-          <t>New: fixes the blocker found by the 14 Oct lifecycle run (owners saw only their newest shop). Checked on test: all 7 shops listed, choice kept after reload, the bakery's orders and rider pickup code shown.</t>
+          <t>Released 15 Oct by #175 (cherry-pick of #168; staging's later changes not included). Live on gokesari.com 14:43 UTC; /shop pages still redirect to sign-in when signed out. Checked on test in the 14 Oct lifecycle run (TR-23).</t>
         </is>
       </c>
       <c r="R214" s="12" t="inlineStr">
@@ -34843,19 +34816,19 @@
         </is>
       </c>
       <c r="F132" s="10" t="n"/>
-      <c r="G132" s="38" t="inlineStr">
-        <is>
-          <t>COMPLETED</t>
-        </is>
-      </c>
-      <c r="H132" s="39" t="inlineStr">
+      <c r="G132" s="10" t="inlineStr">
+        <is>
+          <t>COMPLETED</t>
+        </is>
+      </c>
+      <c r="H132" s="12" t="inlineStr">
         <is>
           <t>#146-#149; #169; #175</t>
         </is>
       </c>
-      <c r="I132" s="39" t="inlineStr">
-        <is>
-          <t>Live on gokesari.com since 15 Oct: the owner's browser reads the photo and pre-fills the details</t>
+      <c r="I132" s="12" t="inlineStr">
+        <is>
+          <t>Photos read in the owner's browser on gokesari.com since 15 Oct (#175); PDFs on the server</t>
         </is>
       </c>
     </row>
@@ -35268,17 +35241,17 @@
       <c r="F143" s="10" t="n"/>
       <c r="G143" s="10" t="inlineStr">
         <is>
-          <t>IN PROGRESS</t>
+          <t>COMPLETED</t>
         </is>
       </c>
       <c r="H143" s="12" t="inlineStr">
         <is>
-          <t>#168</t>
+          <t>#168; #175</t>
         </is>
       </c>
       <c r="I143" s="12" t="inlineStr">
         <is>
-          <t>On test; release to production next</t>
+          <t>Live on gokesari.com since 15 Oct (#175)</t>
         </is>
       </c>
     </row>
@@ -38218,7 +38191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L176"/>
+  <dimension ref="A1:L183"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" outlineLevelRow="0"/>
   <cols>
     <col width="7" customWidth="1" style="1" min="1" max="1"/>
@@ -48356,17 +48329,17 @@
       </c>
       <c r="J170" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>NEW-062</t>
         </is>
       </c>
       <c r="K170" s="12" t="inlineStr">
         <is>
-          <t>Not yet (test site only)</t>
+          <t>#175 (cherry-pick); #177</t>
         </is>
       </c>
       <c r="L170" s="12" t="inlineStr">
         <is>
-          <t>CSP adds 'wasm-unsafe-eval'; switch DOCUMENT_OCR_BROWSER=off goes back to server-only.</t>
+          <t>CSP adds 'wasm-unsafe-eval'; switch DOCUMENT_OCR_BROWSER=off goes back to server-only. Verified on test 15 Oct (TR-26).</t>
         </is>
       </c>
     </row>
@@ -48398,7 +48371,7 @@
       </c>
       <c r="F171" s="12" t="inlineStr">
         <is>
-          <t>Open (draft)</t>
+          <t>Merged</t>
         </is>
       </c>
       <c r="G171" s="12" t="inlineStr">
@@ -48408,7 +48381,7 @@
       </c>
       <c r="H171" s="12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="I171" s="12" t="inlineStr">
@@ -48428,7 +48401,7 @@
       </c>
       <c r="L171" s="12" t="inlineStr">
         <is>
-          <t>Waiting for the owner's 'merge'.</t>
+          <t>Merged by the owner 15 Oct; results, tracker and the morning 15 Oct status report.</t>
         </is>
       </c>
     </row>
@@ -48494,7 +48467,7 @@
         </is>
       </c>
     </row>
-    <row r="173" ht="27" customHeight="1">
+    <row r="173" ht="39" customHeight="1">
       <c r="A173" s="34" t="n">
         <v>172</v>
       </c>
@@ -48505,7 +48478,7 @@
       </c>
       <c r="C173" s="12" t="inlineStr">
         <is>
-          <t>Fix</t>
+          <t>Fix / hotfix</t>
         </is>
       </c>
       <c r="D173" s="12" t="inlineStr">
@@ -48556,187 +48529,595 @@
     </row>
     <row r="174" ht="27" customHeight="1">
       <c r="A174" s="34" t="n">
+        <v>173</v>
+      </c>
+      <c r="B174" s="12" t="inlineStr">
+        <is>
+          <t>Bulk product upload (Excel/CSV) with shop inventory update</t>
+        </is>
+      </c>
+      <c r="C174" s="12" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D174" s="12" t="inlineStr">
+        <is>
+          <t>claude/amazing-ritchie-9vlq9f -&gt; staging</t>
+        </is>
+      </c>
+      <c r="E174" s="12" t="inlineStr">
+        <is>
+          <t>Test site (staging -&gt; test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F174" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G174" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H174" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I174" s="12" t="inlineStr">
+        <is>
+          <t>GS-013</t>
+        </is>
+      </c>
+      <c r="J174" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K174" s="12" t="inlineStr">
+        <is>
+          <t>#179</t>
+        </is>
+      </c>
+      <c r="L174" s="12" t="inlineStr">
+        <is>
+          <t>Migration 0077.</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="27" customHeight="1">
+      <c r="A175" s="34" t="n">
+        <v>174</v>
+      </c>
+      <c r="B175" s="12" t="inlineStr">
+        <is>
+          <t>Bulk product upload: live test run on test.gokesari.com (23/23 pass)</t>
+        </is>
+      </c>
+      <c r="C175" s="12" t="inlineStr">
+        <is>
+          <t>QA / tests</t>
+        </is>
+      </c>
+      <c r="D175" s="12" t="inlineStr">
+        <is>
+          <t>claude/amazing-ritchie-9vlq9f -&gt; staging</t>
+        </is>
+      </c>
+      <c r="E175" s="12" t="inlineStr">
+        <is>
+          <t>Test site (staging -&gt; test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F175" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G175" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H175" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I175" s="12" t="inlineStr">
+        <is>
+          <t>GS-013</t>
+        </is>
+      </c>
+      <c r="J175" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K175" s="12" t="inlineStr">
+        <is>
+          <t>#179</t>
+        </is>
+      </c>
+      <c r="L175" s="12" t="n"/>
+    </row>
+    <row r="176" ht="27" customHeight="1">
+      <c r="A176" s="34" t="n">
+        <v>175</v>
+      </c>
+      <c r="B176" s="12" t="inlineStr">
+        <is>
+          <t>Release: shop switcher (#168) and browser document reading (#169)</t>
+        </is>
+      </c>
+      <c r="C176" s="12" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D176" s="12" t="inlineStr">
+        <is>
+          <t>claude/peaceful-pascal-jai8w2 -&gt; main</t>
+        </is>
+      </c>
+      <c r="E176" s="12" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F176" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G176" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H176" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I176" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J176" s="12" t="inlineStr">
+        <is>
+          <t>NEW-066, NEW-062</t>
+        </is>
+      </c>
+      <c r="K176" s="12" t="inlineStr">
+        <is>
+          <t>Itself (merged to main)</t>
+        </is>
+      </c>
+      <c r="L176" s="12" t="inlineStr">
+        <is>
+          <t>Cherry-picks of #168 and #169 only; live 14:43 UTC. Production checks PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="27" customHeight="1">
+      <c r="A177" s="34" t="n">
+        <v>176</v>
+      </c>
+      <c r="B177" s="12" t="inlineStr">
+        <is>
+          <t>Release: document photos read in the owner's browser (#169, fixes D-18)</t>
+        </is>
+      </c>
+      <c r="C177" s="12" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D177" s="12" t="inlineStr">
+        <is>
+          <t>staging -&gt; main</t>
+        </is>
+      </c>
+      <c r="E177" s="12" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F177" s="12" t="inlineStr">
+        <is>
+          <t>Closed - not merged</t>
+        </is>
+      </c>
+      <c r="G177" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H177" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I177" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J177" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K177" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L177" s="12" t="inlineStr">
+        <is>
+          <t>Closed: staging also carried #168, #171 (migration 0076) and #173 (migration 0077), not approved for release here. Replaced by #177.</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="27" customHeight="1">
+      <c r="A178" s="34" t="n">
+        <v>177</v>
+      </c>
+      <c r="B178" s="12" t="inlineStr">
+        <is>
+          <t>Release: document photos read in the owner's browser (#169, fixes D-18)</t>
+        </is>
+      </c>
+      <c r="C178" s="12" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D178" s="12" t="inlineStr">
+        <is>
+          <t>claude/gracious-einstein-24qjjh -&gt; main</t>
+        </is>
+      </c>
+      <c r="E178" s="12" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F178" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G178" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H178" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I178" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J178" s="12" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="K178" s="12" t="inlineStr">
+        <is>
+          <t>Itself (merged to main)</t>
+        </is>
+      </c>
+      <c r="L178" s="12" t="inlineStr">
+        <is>
+          <t>Same commit as #175's cherry-pick of #169, merged after it: no code change. Production checks 15 Oct (TR-27) PASS.</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="27" customHeight="1">
+      <c r="A179" s="34" t="n">
+        <v>178</v>
+      </c>
+      <c r="B179" s="12" t="inlineStr">
+        <is>
+          <t>Browser document reading (#169): test results on test and production; trackers</t>
+        </is>
+      </c>
+      <c r="C179" s="12" t="inlineStr">
+        <is>
+          <t>Docs / reports</t>
+        </is>
+      </c>
+      <c r="D179" s="12" t="inlineStr">
+        <is>
+          <t>claude/gracious-einstein-24qjjh -&gt; main</t>
+        </is>
+      </c>
+      <c r="E179" s="12" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F179" s="12" t="inlineStr">
+        <is>
+          <t>Open (draft)</t>
+        </is>
+      </c>
+      <c r="G179" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H179" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I179" s="12" t="inlineStr">
+        <is>
+          <t>NEW-062</t>
+        </is>
+      </c>
+      <c r="J179" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K179" s="12" t="inlineStr">
+        <is>
+          <t>Not needed (docs)</t>
+        </is>
+      </c>
+      <c r="L179" s="12" t="inlineStr">
+        <is>
+          <t>Open draft; also edits this workbook and the test tracker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="27" customHeight="1">
+      <c r="A180" s="34" t="n">
+        <v>179</v>
+      </c>
+      <c r="B180" s="12" t="inlineStr">
+        <is>
+          <t>Release: Inventory &amp; Accounting (#171, #172), Bulk product upload (#173, #174); migrations 0076-0078</t>
+        </is>
+      </c>
+      <c r="C180" s="12" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D180" s="12" t="inlineStr">
+        <is>
+          <t>claude/amazing-ritchie-9vlq9f -&gt; main</t>
+        </is>
+      </c>
+      <c r="E180" s="12" t="inlineStr">
+        <is>
+          <t>Production (main -&gt; gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F180" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G180" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="H180" s="12" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="I180" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J180" s="12" t="inlineStr">
+        <is>
+          <t>NEW-067, GS-013</t>
+        </is>
+      </c>
+      <c r="K180" s="12" t="inlineStr">
+        <is>
+          <t>Itself (merged to main)</t>
+        </is>
+      </c>
+      <c r="L180" s="12" t="inlineStr">
+        <is>
+          <t>Migrations 0076-0078 via MIGRATE_ON_BUILD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="39" customHeight="1">
+      <c r="A181" s="34" t="n">
         <v>180</v>
       </c>
-      <c r="B174" s="12" t="inlineStr">
+      <c r="B181" s="12" t="inlineStr">
         <is>
           <t>Release: Inventory &amp; Accounting (#171, #172) + bulk product upload (#173, #174)</t>
         </is>
       </c>
-      <c r="C174" s="12" t="inlineStr">
-        <is>
-          <t>Release</t>
-        </is>
-      </c>
-      <c r="D174" s="12" t="inlineStr">
+      <c r="C181" s="12" t="inlineStr">
+        <is>
+          <t>Release (staging -&gt; main)</t>
+        </is>
+      </c>
+      <c r="D181" s="12" t="inlineStr">
         <is>
           <t>claude/nice-cori-6p1wb2 -&gt; main</t>
         </is>
       </c>
-      <c r="E174" s="12" t="inlineStr">
+      <c r="E181" s="12" t="inlineStr">
         <is>
           <t>Production (main -&gt; gokesari.com)</t>
         </is>
       </c>
-      <c r="F174" s="12" t="inlineStr">
-        <is>
-          <t>Closed (duplicate)</t>
-        </is>
-      </c>
-      <c r="G174" s="12" t="inlineStr">
+      <c r="F181" s="12" t="inlineStr">
+        <is>
+          <t>Closed - not merged</t>
+        </is>
+      </c>
+      <c r="G181" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H174" s="12" t="inlineStr">
+      <c r="H181" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I174" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J174" s="12" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K174" s="12" t="inlineStr">
+      <c r="I181" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J181" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K181" s="12" t="inlineStr">
         <is>
           <t>Superseded by #179</t>
         </is>
       </c>
-      <c r="L174" s="12" t="inlineStr">
-        <is>
-          <t>Same staging code as #179, which merged first; CI was green (preview APK re-run after a corrupt NDK download).</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="40" t="n">
-        <v>176</v>
-      </c>
-      <c r="B175" s="39" t="inlineStr">
-        <is>
-          <t>Release: document photos read in the owner's browser (#169)</t>
-        </is>
-      </c>
-      <c r="C175" s="39" t="inlineStr">
-        <is>
-          <t>Release (staging -&gt; main)</t>
-        </is>
-      </c>
-      <c r="D175" s="39" t="inlineStr">
-        <is>
-          <t>staging -&gt; main</t>
-        </is>
-      </c>
-      <c r="E175" s="39" t="inlineStr">
-        <is>
-          <t>Production (main -&gt; gokesari.com)</t>
-        </is>
-      </c>
-      <c r="F175" s="39" t="inlineStr">
-        <is>
-          <t>Closed - not merged</t>
-        </is>
-      </c>
-      <c r="G175" s="39" t="inlineStr">
+      <c r="L181" s="12" t="inlineStr">
+        <is>
+          <t>Same staging code as #179, which merged first; CI was green (preview APK re-run after a corrupt NDK download). Duplicate of #179.</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="27" customHeight="1">
+      <c r="A182" s="34" t="n">
+        <v>181</v>
+      </c>
+      <c r="B182" s="12" t="inlineStr">
+        <is>
+          <t>Bulk product upload: production results; staging level with main after release #179</t>
+        </is>
+      </c>
+      <c r="C182" s="12" t="inlineStr">
+        <is>
+          <t>Docs / reports</t>
+        </is>
+      </c>
+      <c r="D182" s="12" t="inlineStr">
+        <is>
+          <t>claude/amazing-ritchie-9vlq9f -&gt; staging</t>
+        </is>
+      </c>
+      <c r="E182" s="12" t="inlineStr">
+        <is>
+          <t>Test site (staging -&gt; test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F182" s="12" t="inlineStr">
+        <is>
+          <t>Merged</t>
+        </is>
+      </c>
+      <c r="G182" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H175" s="39" t="inlineStr">
+      <c r="H182" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I175" s="39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J175" s="39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K175" s="39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L175" s="39" t="inlineStr">
-        <is>
-          <t>Closed: staging also carried #168, #171 (migration 0076) and #173 (migration 0077), not approved for release here. Replaced by #177.</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="40" t="n">
-        <v>177</v>
-      </c>
-      <c r="B176" s="39" t="inlineStr">
-        <is>
-          <t>Release: document photos read in the owner's browser (#169, fixes D-18)</t>
-        </is>
-      </c>
-      <c r="C176" s="39" t="inlineStr">
-        <is>
-          <t>Release (branch -&gt; main)</t>
-        </is>
-      </c>
-      <c r="D176" s="39" t="inlineStr">
-        <is>
-          <t>claude/gracious-einstein-24qjjh -&gt; main</t>
-        </is>
-      </c>
-      <c r="E176" s="39" t="inlineStr">
-        <is>
-          <t>Production (main -&gt; gokesari.com)</t>
-        </is>
-      </c>
-      <c r="F176" s="39" t="inlineStr">
+      <c r="I182" s="12" t="inlineStr">
+        <is>
+          <t>GS-013</t>
+        </is>
+      </c>
+      <c r="J182" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K182" s="12" t="inlineStr">
+        <is>
+          <t>Not needed (docs)</t>
+        </is>
+      </c>
+      <c r="L182" s="12" t="n"/>
+    </row>
+    <row r="183" ht="27" customHeight="1">
+      <c r="A183" s="34" t="n">
+        <v>182</v>
+      </c>
+      <c r="B183" s="12" t="inlineStr">
+        <is>
+          <t>Inventory &amp; Accounting: testing report, tracker and 15 Oct status report (after release #179)</t>
+        </is>
+      </c>
+      <c r="C183" s="12" t="inlineStr">
+        <is>
+          <t>Docs / reports</t>
+        </is>
+      </c>
+      <c r="D183" s="12" t="inlineStr">
+        <is>
+          <t>claude/nice-cori-6p1wb2 -&gt; staging</t>
+        </is>
+      </c>
+      <c r="E183" s="12" t="inlineStr">
+        <is>
+          <t>Test site (staging -&gt; test.gokesari.com)</t>
+        </is>
+      </c>
+      <c r="F183" s="12" t="inlineStr">
         <is>
           <t>Merged</t>
         </is>
       </c>
-      <c r="G176" s="39" t="inlineStr">
+      <c r="G183" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="H176" s="39" t="inlineStr">
+      <c r="H183" s="12" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="I176" s="39" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J176" s="39" t="inlineStr">
-        <is>
-          <t>NEW-062</t>
-        </is>
-      </c>
-      <c r="K176" s="39" t="inlineStr">
-        <is>
-          <t>Itself (merged to main)</t>
-        </is>
-      </c>
-      <c r="L176" s="39" t="inlineStr">
-        <is>
-          <t>Same commit as #175's cherry-pick of #169, merged after it: no code change. Production checks 15 Oct (TR-27) PASS.</t>
-        </is>
-      </c>
+      <c r="I183" s="12" t="inlineStr">
+        <is>
+          <t>NEW-067</t>
+        </is>
+      </c>
+      <c r="J183" s="12" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K183" s="12" t="inlineStr">
+        <is>
+          <t>Not needed (docs)</t>
+        </is>
+      </c>
+      <c r="L183" s="12" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L172"/>
-  <conditionalFormatting sqref="F2:F172">
+  <autoFilter ref="A1:L183"/>
+  <conditionalFormatting sqref="F2:F183">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
       <formula>"Merged"</formula>
     </cfRule>
@@ -48922,6 +49303,17 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A170" r:id="rId169"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A171" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A183" r:id="rId182"/>
   </hyperlinks>
   <pageMargins left="0.3" right="0.3" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" paperSize="9" scale="100" fitToHeight="0" fitToWidth="1" firstPageNumber="1" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -50590,7 +50982,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="75" customFormat="1" customHeight="1" s="2">
+    <row r="42" ht="63" customFormat="1" customHeight="1" s="2">
       <c r="A42" s="10" t="n">
         <v>41</v>
       </c>
@@ -50604,7 +50996,7 @@
           <t>Document auto-read engine</t>
         </is>
       </c>
-      <c r="D42" s="39" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Resolved 15 Oct: #169 reads the photo in the owner's browser (no document leaves the device to be read); released to gokesari.com (#175 / #177) and verified on test and production. No decision on Claude for KYC documents is needed. Before: the local OCR worker did not start on Hostinger.</t>
         </is>
@@ -50616,10 +51008,10 @@
       </c>
       <c r="F42" s="12" t="inlineStr">
         <is>
-          <t>Dev (release)</t>
-        </is>
-      </c>
-      <c r="G42" s="39" t="inlineStr">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -50750,7 +51142,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="63" customFormat="1" customHeight="1" s="2">
+    <row r="46" ht="39" customFormat="1" customHeight="1" s="2">
       <c r="A46" s="10" t="n">
         <v>45</v>
       </c>
@@ -50790,7 +51182,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="39" customFormat="1" customHeight="1" s="2">
+    <row r="47" ht="27" customFormat="1" customHeight="1" s="2">
       <c r="A47" s="10" t="n">
         <v>46</v>
       </c>
@@ -50830,167 +51222,167 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="1" t="n">
+    <row r="48" ht="39" customHeight="1">
+      <c r="A48" s="10" t="n">
         <v>47</v>
       </c>
-      <c r="B48" s="1" t="inlineStr">
+      <c r="B48" s="12" t="inlineStr">
         <is>
           <t>Release blocker</t>
         </is>
       </c>
-      <c r="C48" s="1" t="inlineStr">
+      <c r="C48" s="12" t="inlineStr">
         <is>
           <t>Bulk product upload: production checks signed in</t>
         </is>
       </c>
-      <c r="D48" s="1" t="inlineStr">
+      <c r="D48" s="12" t="inlineStr">
         <is>
           <t>Live on gokesari.com since 15 Oct 15:58 UTC (#179). A signed-in import on production needs a designated test shop; the Production database workflow needs its repository variables set.</t>
         </is>
       </c>
-      <c r="E48" s="1" t="inlineStr">
+      <c r="E48" s="12" t="inlineStr">
         <is>
           <t>BPU-16</t>
         </is>
       </c>
-      <c r="F48" s="1" t="inlineStr">
+      <c r="F48" s="12" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="G48" s="1" t="inlineStr">
+      <c r="G48" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="H48" s="1" t="inlineStr">
+      <c r="H48" s="12" t="inlineStr">
         <is>
           <t>docs/product-import-2026-10/README.md</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="1" t="n">
+    <row r="49" ht="27" customHeight="1">
+      <c r="A49" s="10" t="n">
         <v>48</v>
       </c>
-      <c r="B49" s="1" t="inlineStr">
+      <c r="B49" s="12" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="C49" s="1" t="inlineStr">
+      <c r="C49" s="12" t="inlineStr">
         <is>
           <t>Bulk upload: MRP in the file</t>
         </is>
       </c>
-      <c r="D49" s="1" t="inlineStr">
+      <c r="D49" s="12" t="inlineStr">
         <is>
           <t>Stored as the listing MRP (shop_listing_details.mrp_paise); master MRP unchanged; price above it not applied</t>
         </is>
       </c>
-      <c r="E49" s="1" t="inlineStr">
+      <c r="E49" s="12" t="inlineStr">
         <is>
           <t>BPU-03</t>
         </is>
       </c>
-      <c r="F49" s="1" t="inlineStr">
+      <c r="F49" s="12" t="inlineStr">
         <is>
           <t>Dev (recorded)</t>
         </is>
       </c>
-      <c r="G49" s="1" t="inlineStr">
+      <c r="G49" s="12" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
       </c>
-      <c r="H49" s="1" t="inlineStr">
+      <c r="H49" s="12" t="inlineStr">
         <is>
           <t>docs/product-import-2026-10/README.md</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="1" t="n">
+    <row r="50" ht="27" customHeight="1">
+      <c r="A50" s="10" t="n">
         <v>49</v>
       </c>
-      <c r="B50" s="1" t="inlineStr">
+      <c r="B50" s="12" t="inlineStr">
         <is>
           <t>Decision</t>
         </is>
       </c>
-      <c r="C50" s="1" t="inlineStr">
+      <c r="C50" s="12" t="inlineStr">
         <is>
           <t>Bulk upload: uncategorised products</t>
         </is>
       </c>
-      <c r="D50" s="1" t="inlineStr">
+      <c r="D50" s="12" t="inlineStr">
         <is>
           <t>Go to the system category General</t>
         </is>
       </c>
-      <c r="E50" s="1" t="inlineStr">
+      <c r="E50" s="12" t="inlineStr">
         <is>
           <t>BPU-04</t>
         </is>
       </c>
-      <c r="F50" s="1" t="inlineStr">
+      <c r="F50" s="12" t="inlineStr">
         <is>
           <t>Dev (recorded)</t>
         </is>
       </c>
-      <c r="G50" s="1" t="inlineStr">
+      <c r="G50" s="12" t="inlineStr">
         <is>
           <t>Decided</t>
         </is>
       </c>
-      <c r="H50" s="1" t="inlineStr">
+      <c r="H50" s="12" t="inlineStr">
         <is>
           <t>docs/product-import-2026-10/README.md</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" s="1" t="n">
+    <row r="51" ht="27" customHeight="1">
+      <c r="A51" s="10" t="n">
         <v>50</v>
       </c>
-      <c r="B51" s="1" t="inlineStr">
+      <c r="B51" s="12" t="inlineStr">
         <is>
           <t>Go-live blocker</t>
         </is>
       </c>
-      <c r="C51" s="1" t="inlineStr">
+      <c r="C51" s="12" t="inlineStr">
         <is>
           <t>Bulk upload: mobile store builds</t>
         </is>
       </c>
-      <c r="D51" s="1" t="inlineStr">
+      <c r="D51" s="12" t="inlineStr">
         <is>
           <t>EAS / Expo account and Apple Developer account for the AAB and the iPhone build</t>
         </is>
       </c>
-      <c r="E51" s="1" t="inlineStr">
+      <c r="E51" s="12" t="inlineStr">
         <is>
           <t>BPU-10, BPU-11</t>
         </is>
       </c>
-      <c r="F51" s="1" t="inlineStr">
+      <c r="F51" s="12" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
       </c>
-      <c r="G51" s="1" t="inlineStr">
+      <c r="G51" s="12" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
-      <c r="H51" s="1" t="inlineStr">
+      <c r="H51" s="12" t="inlineStr">
         <is>
           <t>docs/product-import-2026-10/README.md</t>
         </is>
       </c>
     </row>
-    <row r="52" ht="63" customHeight="1">
+    <row r="52" ht="51" customHeight="1">
       <c r="A52" s="10" t="n">
         <v>51</v>
       </c>
@@ -51030,7 +51422,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="63" customHeight="1">
+    <row r="53" ht="39" customHeight="1">
       <c r="A53" s="10" t="n">
         <v>52</v>
       </c>
@@ -51070,7 +51462,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="63" customHeight="1">
+    <row r="54" ht="39" customHeight="1">
       <c r="A54" s="10" t="n">
         <v>53</v>
       </c>
@@ -51110,7 +51502,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="63" customHeight="1">
+    <row r="55" ht="27" customHeight="1">
       <c r="A55" s="10" t="n">
         <v>54</v>
       </c>
@@ -51150,7 +51542,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="63" customHeight="1">
+    <row r="56" ht="39" customHeight="1">
       <c r="A56" s="10" t="n">
         <v>55</v>
       </c>
@@ -51190,7 +51582,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="63" customHeight="1">
+    <row r="57" ht="51" customHeight="1">
       <c r="A57" s="10" t="n">
         <v>56</v>
       </c>
@@ -51231,8 +51623,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H47"/>
-  <conditionalFormatting sqref="G2:G47">
+  <autoFilter ref="A1:H57"/>
+  <conditionalFormatting sqref="G2:G57">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="3">
       <formula>"Open"</formula>
     </cfRule>

</xml_diff>